<commit_message>
Atlas em outubro: com --orbe-anterior, as linhas de setembro entram na nota pela taxa confirmada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/outubro/02_tabela_taxas_contratadas.xlsx
+++ b/tests/fixtures/outubro/02_tabela_taxas_contratadas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxas vigentes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANTIGO 2025 - nao usar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Taxas vigentes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ANTIGO 2025 - nao usar" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -494,6 +494,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -692,7 +693,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -776,7 +776,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -817,7 +816,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -858,7 +856,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -945,7 +942,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1059,7 +1055,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1103,7 +1098,6 @@
           <t>01/06/2026</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1147,7 +1141,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1200,7 +1193,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1253,7 +1245,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1294,7 +1285,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1363,7 +1353,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1402,7 +1391,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1446,7 +1434,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1490,7 +1477,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1529,7 +1515,6 @@
           <t>01/06/2026</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1575,7 +1560,6 @@
           <t>01/01/2026</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1619,8 +1603,54 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Atlas Idiomas Ltda</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>39566044000119</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1076801732</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0199</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.0349</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.0449</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.009900000000000001</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>a partir de 10/09/2026</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>DADO SINTÉTICO: contrato confirmado pelo comercial em outubro</t>
+        </is>
+      </c>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>* spread em branco = padrão</t>
         </is>

</xml_diff>